<commit_message>
all done(script cleaning left)
</commit_message>
<xml_diff>
--- a/new_results/output_data.xlsx
+++ b/new_results/output_data.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1388,6 +1388,51 @@
         </is>
       </c>
       <c r="C64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>FRONT</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>TD-M-7537 052924</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>FRONT</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>JUD4105 052824</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>FRONT</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>JUD4106 052824</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1402,7 +1447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1975,6 +2020,96 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TD-M-7537 052924</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>ER</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>OS</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>JUD4105 052824</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>SUM</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>OS</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>5/28/24</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>JUD4106 052824</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>OS</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Done(code optimization left )
</commit_message>
<xml_diff>
--- a/new_results/output_data.xlsx
+++ b/new_results/output_data.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1433,6 +1433,216 @@
         </is>
       </c>
       <c r="C67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>FRONT</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>ECT0261 052924</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>FRONT</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>JUD3151 052924</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>FRONT</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>TDM6599 052924</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>FRONT</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>KAY0823 052924</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>FRONT</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>KAY0921 052924</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>FRONT</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>KAY0921 052924</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>FRONT</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>TDM6161 052924</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>FRONT</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>EHM2463 052924</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>FRONT</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>TDFW2394 052824</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>FRONT</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>TDFW2393 052824</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>FRONT</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>TDFW2396  052824</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>FRONT</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>EIE0711 052824</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>BACK</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>LUN2029X 052924</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>BACK</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2405293370</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1447,7 +1657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2110,6 +2320,418 @@
       </c>
       <c r="H20" t="inlineStr"/>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ECT0261 052924</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>HOL</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>ER</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>OS</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>JUD3151 052924</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>HOL</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>ER</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>OS</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TDM6599 052924</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>HOL</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>ER</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>OS</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>KAY0823 052924</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>HOL</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>ER</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>OS</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>KAY0921 052924</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>HOL</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>ER</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>OS</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>KAY0921 052924</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>HOL</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>ER</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>OS</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TDM6161 052924</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>HOL</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>ER</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>OS</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>EHM2463 052924</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>HOL</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>ER</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>OS</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TDFW2394 052824</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>SUM</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>HAIR</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>TDFW2393 052824</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>SUN</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>TDFW2396  052824</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>HOL</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>EIE0711 052824</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>HOL</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>LUN2029X 052924</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2405293370</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>